<commit_message>
Leads: 2026-10-25 04:44 UTC (cycle 2)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-25.xlsx
+++ b/output/leads_2026-10-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:L3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -563,6 +563,62 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Roofing Davenport Iowa | Free Quotes | Quad Cities Roofing</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>davenportroofingco.us</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>https://davenportroofingco.us/</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Why Davenport</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>darin@landformsusa.com</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Davenport IA</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>76</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>residential roofing company Davenport IA</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-25 04:47 UTC (cycle 4)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-25.xlsx
+++ b/output/leads_2026-10-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -594,7 +594,6 @@
           <t>darin@landformsusa.com</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
           <t>Davenport IA</t>
@@ -614,6 +613,66 @@
         </is>
       </c>
       <c r="L3" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Iowa Heating &amp; Cooling</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>iowaheatingandcooling.work</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>https://iowaheatingandcooling.work/locations/iowa-city/</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Auburn East</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>help@iowaheatingandcooling.work</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>(515) 355-0909</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Iowa City IA</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>100</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>heating and cooling company Iowa City IA</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
         <is>
           <t>2026-10-25</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-25 04:56 UTC (cycle 10)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-25.xlsx
+++ b/output/leads_2026-10-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -678,6 +678,66 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Surf's Up Home Service</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>surfsupservice.com</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>https://www.surfsupservice.com/furnace-repair</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Furnace Failure</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>info@surfsupservice.com</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>(251) 338-9254</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Mobile AL</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>90</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>furnace repair Mobile AL</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-25 04:59 UTC (cycle 12)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-25.xlsx
+++ b/output/leads_2026-10-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -738,6 +738,66 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>T. Conlan Roofing | Best Roofing Services in Jacksonville, Florida</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>tconlanroofing.com</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>https://www.tconlanroofing.com/</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Family Residential</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>estimating@tconlanroofing.com</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>904-661-1591</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Jacksonville FL</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>100</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>roofing contractor Jacksonville FL</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-25 13:07 UTC (cycle 2)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-25.xlsx
+++ b/output/leads_2026-10-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -798,6 +798,66 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>510 Roofing | Expert Roofing Services in Kansas City | Roof Repairs, Replacement</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>510roofingkc.com</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>https://www.510roofingkc.com/</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Honor At</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>sales@510roofingkc.com</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>(913) 300-0421</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Kansas City KS</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>86</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>roof replacement Kansas City KS</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-25 13:08 UTC (cycle 3)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-25.xlsx
+++ b/output/leads_2026-10-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -858,6 +858,66 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Home Comfort Mechanical</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>comfymech.com</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>https://comfymech.com/</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Local Owner</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>g.rodrigue1129@gmail.com</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>(603) 402-6434</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Nashua NH</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>86</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>air conditioning repair Nashua NH</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-25 13:11 UTC (cycle 5)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-25.xlsx
+++ b/output/leads_2026-10-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -918,6 +918,66 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Roof Repair Company Sarasota FL - Residential &amp; Commercial</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>wolffroofing.com</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>https://www.wolffroofing.com/roof-repairs</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Poor Maintenance</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>contact@wolffroofing.com</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>941-920-1805</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Sarasota FL</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>100</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>roof repair company Sarasota FL</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-25 13:14 UTC (cycle 7)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-25.xlsx
+++ b/output/leads_2026-10-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:L10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -978,6 +978,66 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Plumbers in Colorado Springs | Incline Plumbing LLC</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>inclineplumbing.com</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>https://www.inclineplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Colorado Springs</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>inclineplumbinganddrain@gmail.com</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>(719) 922-3350</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Colorado Springs CO</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>90</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>plumber Colorado Springs CO</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-25 13:17 UTC (cycle 9)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-25.xlsx
+++ b/output/leads_2026-10-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1038,6 +1038,66 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>AMAYA ROOFING</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>amayaroofinginc.com</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>https://www.amayaroofinginc.com/</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>At Amaya</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>sales@amayaroofinginc.com</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>702-420-2419</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Las Vegas NV</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>100</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>roofer Las Vegas NV</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-25 13:18 UTC (cycle 10)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-25.xlsx
+++ b/output/leads_2026-10-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:L12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1098,6 +1098,66 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>BlueCool AC Repair Services</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>bluecoolacrepair.com</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>https://bluecoolacrepair.com/air-conditioning-repair-in-pembroke-pines-fl/</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Team The</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>info@bluecoolacrepair.com</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>(645) 237-1292</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Pembroke Pines FL</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>90</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>air conditioning repair Pembroke Pines FL</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-25 13:23 UTC (cycle 13)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-25.xlsx
+++ b/output/leads_2026-10-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L12"/>
+  <dimension ref="A1:L16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1158,6 +1158,242 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Orlando Air Conditioning Experts</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>orlandoairconditioningexperts.com</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>https://orlandoairconditioningexperts.com/</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>eben@eyebytes.com</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>(407) 986-9977</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Orlando FL</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>98</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>AC installation Orlando FL</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Blue Collar Contracting | Trusted Exterior Services in Kansas City</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>bluecollarcontractingkc.com</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>https://bluecollarcontractingkc.com/olathe/</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Kansas City</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>dylan@bluecollarroofing.org</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>816-810-9251</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Olathe KS</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>90</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>roofing contractor Olathe KS</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>rufplus.com</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>rufplus.com</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>https://rufplus.com/roofing-contractor-olathe-ks/</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Picked Expertise</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>angel@rufplus.com</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>(877) 783-4648</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Olathe KS</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>90</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>roofing contractor Olathe KS</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>AirPlus, Inc</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>airplusct.com</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>https://www.airplusct.com/</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>President Meet</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>office@airplusinc.net</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>(203) 854-9751</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Norwalk CT</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
+        <v>88</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>air conditioning repair Norwalk CT</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-25 13:24 UTC (cycle 14)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-25.xlsx
+++ b/output/leads_2026-10-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L16"/>
+  <dimension ref="A1:L17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1179,7 +1179,6 @@
           <t>https://orlandoairconditioningexperts.com/</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
           <t>eben@eyebytes.com</t>
@@ -1389,6 +1388,66 @@
         </is>
       </c>
       <c r="L16" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>River City Sewers, LLC</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>rivercitysewersllc.com</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>https://rivercitysewersllc.com/</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Know Who</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>rivercitysewersllc@gmail.com</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>(316) 235-9046</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Wichita KS</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
+        <v>84</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>sewer repair Wichita KS</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
         <is>
           <t>2026-10-25</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-25 18:49 UTC (cycle 1)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-25.xlsx
+++ b/output/leads_2026-10-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L17"/>
+  <dimension ref="A1:L18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1453,6 +1453,66 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Superior Plumbing</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>superiorplumbing.net</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>https://superiorplumbing.net/drain-cleaning/</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Professional Drain</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>aasuperiorplumbing@gmail.com</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>408.446.1760</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>San Jose CA</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
+        <v>100</v>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>drain cleaning service San Jose CA</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-25 18:51 UTC (cycle 2)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-25.xlsx
+++ b/output/leads_2026-10-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L18"/>
+  <dimension ref="A1:L20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1513,6 +1513,118 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Emergency Plumbing Boise, ID | Goodson Plumbing Services</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>robgoodsonplumbing.com</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>https://www.robgoodsonplumbing.com/emergency-plumbing-service</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>michelle@robgoodsonplumbing.com</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>(208) 629-4278</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Boise ID</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
+        <v>94</v>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>emergency plumber Boise ID</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Scott Smith Roofing</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>scottsmithroofing.com</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>https://www.scottsmithroofing.com/</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>superiorseptic1@gmail.com</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>352-867-0044</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Ocala FL</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
+        <v>88</v>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>roof repair company Ocala FL</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-25 18:55 UTC (cycle 5)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-25.xlsx
+++ b/output/leads_2026-10-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L20"/>
+  <dimension ref="A1:L21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1534,7 +1534,6 @@
           <t>https://www.robgoodsonplumbing.com/emergency-plumbing-service</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr">
         <is>
           <t>michelle@robgoodsonplumbing.com</t>
@@ -1590,7 +1589,6 @@
           <t>https://www.scottsmithroofing.com/</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr">
         <is>
           <t>superiorseptic1@gmail.com</t>
@@ -1620,6 +1618,66 @@
         </is>
       </c>
       <c r="L20" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Water Heater Repair Katy TX</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>repairwaterheaterkaty.com</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>https://repairwaterheaterkaty.com/</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Water Heater</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>service@repairwaterheaterkaty.com</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>281-742-0561</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Katy TX</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
+        <v>100</v>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>water heater repair Katy TX</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
         <is>
           <t>2026-10-25</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-25 18:56 UTC (cycle 6)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-25.xlsx
+++ b/output/leads_2026-10-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L21"/>
+  <dimension ref="A1:L22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1683,6 +1683,66 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>ASAP Roofing &amp; Exteriors</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>asaproofingandexteriors.com</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>https://asaproofingandexteriors.com/residential-roofing</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Flat Roofs</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>amuniz@asaproofingandexteriors.com</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>(301) 281-7150</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Washington DC</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
+        <v>90</v>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>residential roofing company Washington DC</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-25 18:58 UTC (cycle 7)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-25.xlsx
+++ b/output/leads_2026-10-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L22"/>
+  <dimension ref="A1:L23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1743,6 +1743,66 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Texas Roofing Project</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>txroofingproject.com</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>https://txroofingproject.com/service-areas/mesquite-tx/</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Professional Roofing</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>info@txroofingproject.com</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>214-600-7661</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Mesquite TX</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
+        <v>100</v>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>roofing contractor Mesquite TX</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-25 18:59 UTC (cycle 8)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-25.xlsx
+++ b/output/leads_2026-10-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L23"/>
+  <dimension ref="A1:L24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1803,6 +1803,66 @@
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>A&amp;E Home Improvement</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>aehomenh.com</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>https://www.aehomenh.com/services/roofing/concord</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Contractor New</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>info@aehomenh.com</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>603-455-0221</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Concord NH</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
+        <v>90</v>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>residential roofing company Concord NH</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-25 19:05 UTC (cycle 12)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-25.xlsx
+++ b/output/leads_2026-10-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L24"/>
+  <dimension ref="A1:L25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1863,6 +1863,66 @@
         </is>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>The Expert Co</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>theexpertco.com</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>https://www.theexpertco.com/roof-repair-minneapolis/</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Local Business</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>office@theexpertcompany.net</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>(952) 393-0060</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Minneapolis MN</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
+        <v>90</v>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>roof repair company Minneapolis MN</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-25 19:07 UTC (cycle 13)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-25.xlsx
+++ b/output/leads_2026-10-25.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L25"/>
+  <dimension ref="A1:L26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1923,6 +1923,66 @@
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Trusted Roofing Contractor in Iowa City | Michel Cuevas Home Improvement</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>michelcuevashome.com</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>https://www.michelcuevashome.com/</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Free Estimates</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>micuevas1986@gmail.com</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>(319) 333-5046</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Iowa City IA</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
+        <v>100</v>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>residential roofing company Iowa City IA</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>